<commit_message>
Clear sample data and history
</commit_message>
<xml_diff>
--- a/bases_movimentacoes.xlsx
+++ b/bases_movimentacoes.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -469,38 +469,6 @@
           <t>observacoes</t>
         </is>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>2026-05-05</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>TMG BASE SORRISO</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>LUVA NITRILICA</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Entrada</t>
-        </is>
-      </c>
-      <c r="E2" t="n">
-        <v>10</v>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>LEANDRO BARRETO</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Repair empty data schemas
</commit_message>
<xml_diff>
--- a/bases_movimentacoes.xlsx
+++ b/bases_movimentacoes.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:G1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -460,11 +460,6 @@
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>origem_destino</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>observacoes</t>
         </is>

</xml_diff>